<commit_message>
Rename and modify rate input files to align with the process names
</commit_message>
<xml_diff>
--- a/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
+++ b/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\EV_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8EEB33-1DAA-4504-840A-7D30D371142C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08ACF175-E6A0-4DD8-9050-EB360FEB9CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -366,9 +366,6 @@
     <t>ODYM_Tutorial6_FabricationYieldLossLL</t>
   </si>
   <si>
-    <t>ODYM_Tutorial6_RemeltingYieldLL</t>
-  </si>
-  <si>
     <t>ODYM_Tutorial6_SectorSplitLL</t>
   </si>
   <si>
@@ -417,21 +414,6 @@
     <t>Share of flow after use going to used export. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
   </si>
   <si>
-    <t>Share of flow after use going to recycling. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
-  </si>
-  <si>
-    <t>ODYM_T6_ToRecyclingRateLL</t>
-  </si>
-  <si>
-    <t>ODYM_T6_ScrapToRefurbishmentRateLL</t>
-  </si>
-  <si>
-    <t>Share of scrap flow after use going to refurbishment. Index structure and Aspect order match based on RemeltingYield as these rates share the same process.</t>
-  </si>
-  <si>
-    <t>Share of input scrap that is recovered as secondary material and goes to recycling.</t>
-  </si>
-  <si>
     <t>38ed7154-01c2-4d21-8128-df10bbd150a6</t>
   </si>
   <si>
@@ -490,6 +472,24 @@
   </si>
   <si>
     <t>Previous process numbering: 0 Environment</t>
+  </si>
+  <si>
+    <t>ODYM_T6_ToSortingRateLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_SortingToRefurbishmentRateLL</t>
+  </si>
+  <si>
+    <t>Share of flow recovered from sorting and goes to recycling.</t>
+  </si>
+  <si>
+    <t>Share of flow after use going to Sorting. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>Share of flow after sorting going to refurbishment. Index structure and Aspect order match based on RemeltingYield as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>ODYM_T6_SortingToRecyclingRateLL</t>
   </si>
 </sst>
 </file>
@@ -1302,7 +1302,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
@@ -1310,7 +1310,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
@@ -1357,7 +1357,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J10" s="13"/>
     </row>
@@ -1435,7 +1435,7 @@
         <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H16" s="21" t="s">
         <v>23</v>
@@ -1458,7 +1458,7 @@
         <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>75</v>
@@ -1481,7 +1481,7 @@
         <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>24</v>
@@ -1666,7 +1666,7 @@
         <v>84</v>
       </c>
       <c r="F28" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
@@ -1680,7 +1680,7 @@
         <v>54</v>
       </c>
       <c r="F29" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
@@ -1688,13 +1688,13 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E30" t="s">
         <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.3">
@@ -1702,13 +1702,13 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E31" t="s">
         <v>54</v>
       </c>
       <c r="F31" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.3">
@@ -1716,13 +1716,13 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E32" t="s">
         <v>55</v>
       </c>
       <c r="F32" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.3">
@@ -1730,13 +1730,13 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E33" t="s">
         <v>54</v>
       </c>
       <c r="F33" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.3">
@@ -1744,13 +1744,13 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E34" t="s">
         <v>54</v>
       </c>
       <c r="F34" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.3">
@@ -1758,13 +1758,13 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E35" t="s">
         <v>54</v>
       </c>
       <c r="F35" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.3">
@@ -1772,13 +1772,13 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E36" t="s">
         <v>55</v>
       </c>
       <c r="F36" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.3">
@@ -1820,7 +1820,7 @@
         <v>108</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E40" t="s">
         <v>94</v>
@@ -1840,10 +1840,10 @@
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C41" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" t="s">
         <v>116</v>
-      </c>
-      <c r="D41" t="s">
-        <v>117</v>
       </c>
       <c r="E41" t="s">
         <v>94</v>
@@ -1886,10 +1886,10 @@
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="D43" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="E43" t="s">
         <v>94</v>
@@ -1909,7 +1909,7 @@
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="44" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D44" s="45"/>
       <c r="E44" s="45" t="s">
@@ -1930,10 +1930,10 @@
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="D45" t="s">
         <v>124</v>
-      </c>
-      <c r="D45" t="s">
-        <v>125</v>
       </c>
       <c r="E45" t="s">
         <v>94</v>
@@ -1948,15 +1948,15 @@
         <v>31</v>
       </c>
       <c r="I45" s="41" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D46" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E46" t="s">
         <v>94</v>
@@ -1971,15 +1971,15 @@
         <v>31</v>
       </c>
       <c r="I46" s="41" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C47" s="27" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D47" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="E47" t="s">
         <v>94</v>
@@ -1994,15 +1994,15 @@
         <v>31</v>
       </c>
       <c r="I47" s="41" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C48" s="27" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="D48" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="E48" t="s">
         <v>94</v>
@@ -2017,15 +2017,15 @@
         <v>31</v>
       </c>
       <c r="I48" s="43" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C49" s="44" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D49" s="45" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E49" s="45" t="s">
         <v>94</v>
@@ -2040,7 +2040,7 @@
         <v>31</v>
       </c>
       <c r="I49" s="46" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Renaming files to remove LL and tutorial 6 from their names (replace with EV and T6 respectively)
</commit_message>
<xml_diff>
--- a/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
+++ b/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\EV_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08ACF175-E6A0-4DD8-9050-EB360FEB9CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43280F3-9D58-4E51-82BB-FAE7D02FE6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="153">
   <si>
     <t>Description</t>
   </si>
@@ -360,18 +360,6 @@
     <t>10_World_Regions</t>
   </si>
   <si>
-    <t>ODYM_Tutorial6_LifetimeLL</t>
-  </si>
-  <si>
-    <t>ODYM_Tutorial6_FabricationYieldLossLL</t>
-  </si>
-  <si>
-    <t>ODYM_Tutorial6_SectorSplitLL</t>
-  </si>
-  <si>
-    <t>ODYM_Classifications_LL</t>
-  </si>
-  <si>
     <t>[310:324)</t>
   </si>
   <si>
@@ -381,9 +369,6 @@
     <t>Scenario analysis of dispersion of EV LIBs.</t>
   </si>
   <si>
-    <t>ODYM_Tutorial6_EVConsumptionLL</t>
-  </si>
-  <si>
     <t>Final consumption of EVs, exogenous model driver</t>
   </si>
   <si>
@@ -490,6 +475,24 @@
   </si>
   <si>
     <t>ODYM_T6_SortingToRecyclingRateLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecyclingSectorSplitLL</t>
+  </si>
+  <si>
+    <t>Distribution of goods after recycling. Based on ODYM_Tutorial6_SectorSplitLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecycledProductsYieldLossLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_EVConsumptionLL</t>
+  </si>
+  <si>
+    <t>ODYM_Classifications_EV</t>
+  </si>
+  <si>
+    <t>ODYM_T6_LifetimeEV</t>
   </si>
 </sst>
 </file>
@@ -1265,7 +1268,7 @@
   <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.77734375" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="3" max="3" width="40.109375" customWidth="1"/>
     <col min="4" max="4" width="44.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.6640625" customWidth="1"/>
     <col min="6" max="6" width="24.77734375" bestFit="1" customWidth="1"/>
@@ -1302,7 +1305,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
@@ -1310,7 +1313,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
@@ -1357,7 +1360,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>111</v>
+        <v>151</v>
       </c>
       <c r="J10" s="13"/>
     </row>
@@ -1435,7 +1438,7 @@
         <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H16" s="21" t="s">
         <v>23</v>
@@ -1458,7 +1461,7 @@
         <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>75</v>
@@ -1481,7 +1484,7 @@
         <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>24</v>
@@ -1666,7 +1669,7 @@
         <v>84</v>
       </c>
       <c r="F28" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
@@ -1680,7 +1683,7 @@
         <v>54</v>
       </c>
       <c r="F29" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
@@ -1688,13 +1691,13 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E30" t="s">
         <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.3">
@@ -1702,13 +1705,13 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E31" t="s">
         <v>54</v>
       </c>
       <c r="F31" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.3">
@@ -1716,13 +1719,13 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E32" t="s">
         <v>55</v>
       </c>
       <c r="F32" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.3">
@@ -1730,13 +1733,13 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E33" t="s">
         <v>54</v>
       </c>
       <c r="F33" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.3">
@@ -1744,13 +1747,13 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E34" t="s">
         <v>54</v>
       </c>
       <c r="F34" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.3">
@@ -1758,13 +1761,13 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E35" t="s">
         <v>54</v>
       </c>
       <c r="F35" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.3">
@@ -1772,13 +1775,13 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E36" t="s">
         <v>55</v>
       </c>
       <c r="F36" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.3">
@@ -1817,10 +1820,10 @@
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
-        <v>108</v>
+        <v>152</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E40" t="s">
         <v>94</v>
@@ -1840,10 +1843,10 @@
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C41" s="27" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="D41" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E41" t="s">
         <v>94</v>
@@ -1863,7 +1866,7 @@
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C42" s="27" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="D42" t="s">
         <v>101</v>
@@ -1886,10 +1889,10 @@
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D43" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E43" t="s">
         <v>94</v>
@@ -1909,9 +1912,11 @@
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="D44" s="45"/>
+        <v>147</v>
+      </c>
+      <c r="D44" s="45" t="s">
+        <v>148</v>
+      </c>
       <c r="E44" s="45" t="s">
         <v>94</v>
       </c>
@@ -1930,10 +1935,10 @@
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D45" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E45" t="s">
         <v>94</v>
@@ -1948,15 +1953,15 @@
         <v>31</v>
       </c>
       <c r="I45" s="41" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="27" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D46" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E46" t="s">
         <v>94</v>
@@ -1971,15 +1976,15 @@
         <v>31</v>
       </c>
       <c r="I46" s="41" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C47" s="27" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E47" t="s">
         <v>94</v>
@@ -1994,15 +1999,15 @@
         <v>31</v>
       </c>
       <c r="I47" s="41" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C48" s="27" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E48" t="s">
         <v>94</v>
@@ -2017,15 +2022,15 @@
         <v>31</v>
       </c>
       <c r="I48" s="43" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C49" s="44" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D49" s="45" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E49" s="45" t="s">
         <v>94</v>
@@ -2040,7 +2045,7 @@
         <v>31</v>
       </c>
       <c r="I49" s="46" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added files and edited code pertinent to the addition of remaining flows out of the recycling process
</commit_message>
<xml_diff>
--- a/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
+++ b/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model_3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\EV_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43280F3-9D58-4E51-82BB-FAE7D02FE6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CDD2E4-48C1-420E-AB4C-82B95C78B631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="164">
   <si>
     <t>Description</t>
   </si>
@@ -493,6 +493,39 @@
   </si>
   <si>
     <t>ODYM_T6_LifetimeEV</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecyclingToBlackMassExport</t>
+  </si>
+  <si>
+    <t>a3e33053-ab7a-4979-be82-d14c6e5eeceh</t>
+  </si>
+  <si>
+    <t>a3e33053-ab7a-4979-be82-d14c6e5eeceg</t>
+  </si>
+  <si>
+    <t>Distribution of after recycling going to black mass exports. Based on ODYM_Tutorial6_SectorSplitLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecyclingToOtherProduction</t>
+  </si>
+  <si>
+    <t>Distribution of after recycling going to other (non EV LIB) production. Based on ODYM_Tutorial6_SectorSplitLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecyclingToRecycledMaterialExport</t>
+  </si>
+  <si>
+    <t>Distribution of after recycling going to recycled material exports. Based on ODYM_Tutorial6_SectorSplitLL</t>
+  </si>
+  <si>
+    <t>a3e33053-ab7a-4979-be82-d14c6e5eecei</t>
+  </si>
+  <si>
+    <t>a3e33053-ab7a-4979-be82-d14c6e5eecej</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RecyclingToDomesticProduction</t>
   </si>
 </sst>
 </file>
@@ -572,7 +605,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -606,6 +639,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -712,7 +751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -800,6 +839,12 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1264,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J63"/>
+  <dimension ref="B2:K70"/>
   <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.77734375" customWidth="1"/>
@@ -1866,171 +1911,171 @@
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C42" s="27" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>101</v>
+        <v>144</v>
       </c>
       <c r="E42" t="s">
         <v>94</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="G42" t="s">
+      <c r="G42" s="40" t="s">
         <v>78</v>
       </c>
       <c r="H42" t="s">
         <v>31</v>
       </c>
-      <c r="I42" s="37" t="s">
-        <v>100</v>
+      <c r="I42" s="41" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="D43" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="E43" t="s">
         <v>94</v>
       </c>
-      <c r="F43" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="G43" s="42" t="s">
-        <v>83</v>
-      </c>
-      <c r="H43" s="42" t="s">
+      <c r="F43" s="40" t="s">
+        <v>97</v>
+      </c>
+      <c r="G43" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="H43" t="s">
         <v>31</v>
       </c>
-      <c r="I43" s="43" t="s">
-        <v>102</v>
+      <c r="I43" s="41" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C44" s="44" t="s">
-        <v>147</v>
-      </c>
-      <c r="D44" s="45" t="s">
-        <v>148</v>
-      </c>
-      <c r="E44" s="45" t="s">
+      <c r="C44" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44" t="s">
+        <v>119</v>
+      </c>
+      <c r="E44" t="s">
         <v>94</v>
       </c>
-      <c r="F44" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="G44" s="45" t="s">
-        <v>83</v>
-      </c>
-      <c r="H44" s="45" t="s">
+      <c r="F44" s="40" t="s">
+        <v>97</v>
+      </c>
+      <c r="G44" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="H44" t="s">
         <v>31</v>
       </c>
-      <c r="I44" s="46" t="s">
-        <v>104</v>
+      <c r="I44" s="41" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D45" t="s">
-        <v>119</v>
+        <v>145</v>
       </c>
       <c r="E45" t="s">
         <v>94</v>
       </c>
-      <c r="F45" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="G45" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="H45" t="s">
+      <c r="F45" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="G45" s="42" t="s">
+        <v>83</v>
+      </c>
+      <c r="H45" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="I45" s="41" t="s">
-        <v>115</v>
+      <c r="I45" s="43" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="27" t="s">
-        <v>114</v>
+        <v>146</v>
       </c>
       <c r="D46" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="E46" t="s">
         <v>94</v>
       </c>
-      <c r="F46" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="G46" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="H46" t="s">
+      <c r="F46" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="G46" s="42" t="s">
+        <v>83</v>
+      </c>
+      <c r="H46" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="I46" s="41" t="s">
-        <v>116</v>
+      <c r="I46" s="43" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C47" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="D47" t="s">
-        <v>144</v>
-      </c>
-      <c r="E47" t="s">
+      <c r="C47" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="D47" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="E47" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="F47" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="G47" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="H47" t="s">
+      <c r="F47" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="G47" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="H47" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="I47" s="41" t="s">
-        <v>117</v>
+      <c r="I47" s="46" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C48" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="D48" t="s">
-        <v>145</v>
-      </c>
-      <c r="E48" t="s">
+      <c r="C48" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="D48" s="51" t="s">
+        <v>148</v>
+      </c>
+      <c r="E48" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="F48" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="G48" s="42" t="s">
+      <c r="F48" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="G48" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="H48" s="42" t="s">
+      <c r="H48" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="I48" s="43" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="I48" s="52" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C49" s="44" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="D49" s="45" t="s">
-        <v>123</v>
+        <v>156</v>
       </c>
       <c r="E49" s="45" t="s">
         <v>94</v>
@@ -2045,77 +2090,202 @@
         <v>31</v>
       </c>
       <c r="I49" s="46" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B51" s="18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="50" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C50" s="44" t="s">
+        <v>157</v>
+      </c>
+      <c r="D50" s="45" t="s">
+        <v>158</v>
+      </c>
+      <c r="E50" s="45" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="G50" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="H50" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="I50" s="46" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="51" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C51" s="44" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51" s="45" t="s">
+        <v>160</v>
+      </c>
+      <c r="E51" s="45" t="s">
+        <v>94</v>
+      </c>
+      <c r="F51" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="G51" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="H51" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="I51" s="46" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="52" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C52" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52" s="45" t="s">
+        <v>158</v>
+      </c>
+      <c r="E52" s="45" t="s">
+        <v>94</v>
+      </c>
+      <c r="F52" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="G52" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="H52" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="I52" s="46" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="53" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C53" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="D53" t="s">
+        <v>101</v>
+      </c>
+      <c r="E53" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53" t="s">
+        <v>97</v>
+      </c>
+      <c r="G53" t="s">
+        <v>78</v>
+      </c>
+      <c r="H53" t="s">
+        <v>31</v>
+      </c>
+      <c r="I53" s="37" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B54" s="48"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="48"/>
+      <c r="E54" s="48"/>
+      <c r="F54" s="48"/>
+      <c r="G54" s="48"/>
+      <c r="H54" s="48"/>
+      <c r="I54" s="49"/>
+      <c r="J54" s="48"/>
+      <c r="K54" s="48"/>
+    </row>
+    <row r="55" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B55" s="48"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="48"/>
+      <c r="E55" s="48"/>
+      <c r="F55" s="48"/>
+      <c r="G55" s="48"/>
+      <c r="H55" s="48"/>
+      <c r="I55" s="49"/>
+      <c r="J55" s="48"/>
+      <c r="K55" s="48"/>
+    </row>
+    <row r="56" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C56" s="47"/>
+      <c r="D56" s="48"/>
+      <c r="E56" s="48"/>
+      <c r="F56" s="48"/>
+      <c r="G56" s="48"/>
+      <c r="H56" s="48"/>
+      <c r="I56" s="49"/>
+    </row>
+    <row r="58" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B58" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C51" s="19"/>
-      <c r="D51" s="19"/>
-      <c r="E51" s="19"/>
-      <c r="F51" s="19"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="20"/>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C52" t="s">
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="20"/>
+    </row>
+    <row r="59" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C59" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C53" s="27" t="s">
+    <row r="60" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C60" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D53" s="33" t="s">
+      <c r="D60" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E60" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="33"/>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D55" s="33"/>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D56" s="33"/>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D57" s="33"/>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D58" s="33"/>
-    </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B60" s="18" t="s">
+    <row r="61" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="D61" s="33"/>
+    </row>
+    <row r="62" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="D62" s="33"/>
+    </row>
+    <row r="63" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="D63" s="33"/>
+    </row>
+    <row r="64" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="D64" s="33"/>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D65" s="33"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B67" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="20"/>
-    </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C61" t="s">
+      <c r="C67" s="19"/>
+      <c r="D67" s="19"/>
+      <c r="E67" s="19"/>
+      <c r="F67" s="19"/>
+      <c r="G67" s="19"/>
+      <c r="H67" s="20"/>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C68" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B63" s="18" t="s">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B70" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="F63" s="19"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="20"/>
+      <c r="C70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>